<commit_message>
Extended procurement report fields
</commit_message>
<xml_diff>
--- a/Сравнение_КП_959777517.xlsx
+++ b/Сравнение_КП_959777517.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Заключение" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сравнение КП'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сравнение КП'!$A$1:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Позиции КП'!$A$1:$H$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Конкурентная карта'!$A$1:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Итоги поставщиков'!$A$1:$E$4</definedName>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,12 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,6 +517,31 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Условия оплаты</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Гарантия</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Срок действия КП</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Страна</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Комментарий</t>
         </is>
       </c>
@@ -522,12 +552,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>120 048,30</t>
+          <t>122 072,00 ₽</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -537,17 +567,42 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>самовывоз</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>от 5 до 7 раб.дн.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>полная оплата счета, акцепт в течение 3 рабочих дней</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>срок резервирования товара 3 рабочих дня</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Оплата означает согласие с условиями поставки. Товар отпускается по факту прихода денег. Уведомление об оплате обязательно.</t>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>3 рабочих дня с даты выставления счета (26 марта 2026 года)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>ACCKee, BESTE</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Доставка - самовывоз из г. Челябинск, ул. Комарова, д. 110. Гарантия не указана. Срок поставки от 5 до 7 рабочих дней. Оплата полная, акцепт оферты в течение 3 рабочих дней.</t>
         </is>
       </c>
     </row>
@@ -557,12 +612,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>122 072,00 ₽</t>
+          <t>120 048,30</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -572,17 +627,42 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>самовывоз</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>от 5 до 7 раб.дн.</t>
+          <t>срок резервирования товара 3 рабочих дня</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Доставка самовывозом из г. Челябинск, ул. Комарова, д. 110. Срок поставки указан для всех позиций от 5 до 7 рабочих дней. НДС включён, сумма НДС 22 012,98 ₽.</t>
+          <t>товар отпускается по факту прихода денег на р/с Поставщика</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>ACCKee</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Оплата означает согласие с условиями поставки. Уведомление об оплате обязательно. Гарантия и срок действия КП не указаны. Доставка не указана.</t>
         </is>
       </c>
     </row>
@@ -607,22 +687,47 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>самовывоз</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>счет действителен 7 календарных дней</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Оплата означает согласие с условиями поставки. Товар отпускается по факту прихода денег на р/с поставщика, при наличии доверенности и паспорта. Срок поставки не указан явно.</t>
+          <t>оплата по факту прихода денег на р/с Поставщика</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>7 календарных дней</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Доставка не указана, гарантия не указана, производитель и страна не указаны.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:L4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -691,12 +796,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -706,7 +811,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB3-TWN3242-43 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB3-TWN3242-43 bh00018</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -721,24 +826,24 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2720,11</t>
+          <t>5205,00</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2720,11</t>
+          <t>5205,00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -748,7 +853,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB3-205 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB3-205 sh00098</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -763,34 +868,34 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>9995,48</t>
+          <t>19127,00</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>9995,48</t>
+          <t>19127,00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>CKB4-TWN4154-50</t>
+          <t>BT50-45</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB4-TWN4154-50 "ACCKee"</t>
+          <t>BESTE Штревель BT50-45 AC00601921</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -800,39 +905,39 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2969,18</t>
+          <t>931,00</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2969,18</t>
+          <t>2793,00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>CKB5-TWN5372-60</t>
+          <t>CKB4-TWN4154-50</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB5-TWN5372-60 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB4-TWN4154-50 bh00015</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -847,34 +952,34 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>3774,23</t>
+          <t>5682,00</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>3774,23</t>
+          <t>5682,00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB5-245</t>
+          <t>CKB5-TWN5372-60</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB5-245 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB5-TWN5372-60 bh00001</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -889,34 +994,34 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>10406,27</t>
+          <t>5883,00</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>10406,27</t>
+          <t>5883,00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB5-165</t>
+          <t>BT50-CKB6-285</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB5-165 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB6-285 db01991</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -931,34 +1036,34 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>8900,10</t>
+          <t>21498,00</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>8900,10</t>
+          <t>21498,00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN115150-75</t>
+          <t>BT50-CKB1-165</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN115150-75 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB1-165 sh00095</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -973,34 +1078,34 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>8529,30</t>
+          <t>16134,00</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>8529,30</t>
+          <t>16134,00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-165</t>
+          <t>CKB6-TWN115150-75</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-165 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB6-TWN115150-75 bh00003</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1015,34 +1120,34 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>8900,10</t>
+          <t>17180,00</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>8900,10</t>
+          <t>17180,00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-285</t>
+          <t>BT50-CKB6-165</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-285 ACCKee</t>
+          <t>ACCKee Оправка BT50-CKB6-165 sh00023</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1057,24 +1162,24 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>13966,30</t>
+          <t>17927,00</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>13966,30</t>
+          <t>17927,00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1084,7 +1189,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN89120-75 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB6-TWN89120-75 bh00002</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1099,12 +1204,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>5283,82</t>
+          <t>10643,00</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>5283,82</t>
+          <t>10643,00</t>
         </is>
       </c>
     </row>
@@ -1121,12 +1226,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-205</t>
+          <t>CKB3-TWN3242-43</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-205 "ACCKee"</t>
+          <t>Расточная головка CKB3-TWN3242-43 "ACCKee"</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1141,12 +1246,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>10406,27</t>
+          <t>2720,11</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>10406,27</t>
+          <t>2720,11</t>
         </is>
       </c>
     </row>
@@ -1163,12 +1268,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN6890-75</t>
+          <t>BT50-CKB3-205</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN6890-75 "ACCKee"</t>
+          <t>Оправка для расточных головок BT50-CKB3-205 "ACCKee"</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1183,12 +1288,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>5032,21</t>
+          <t>9995,48</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>5032,21</t>
+          <t>9995,48</t>
         </is>
       </c>
     </row>
@@ -1205,12 +1310,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-125</t>
+          <t>CKB4-TWN4154-50</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-125 "ACCKee"</t>
+          <t>Расточная головка CKB4-TWN4154-50 "ACCKee"</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1225,12 +1330,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>7667,77</t>
+          <t>2969,18</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>7667,77</t>
+          <t>2969,18</t>
         </is>
       </c>
     </row>
@@ -1247,12 +1352,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-245</t>
+          <t>CKB5-TWN5372-60</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-245 "ACCKee"</t>
+          <t>Расточная головка CKB5-TWN5372-60 "ACCKee"</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1267,12 +1372,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>11090,89</t>
+          <t>3774,23</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>11090,89</t>
+          <t>3774,23</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1394,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB4-245</t>
+          <t>BT50-CKB5-245</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB4-245 "ACCKee"</t>
+          <t>Оправка для расточных головок BT50-CKB5-245 "ACCKee"</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1321,22 +1426,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>CKB3-TWN3242-43</t>
+          <t>BT50-CKB5-165</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB3-TWN3242-43 bh00018</t>
+          <t>Оправка для расточных головок BT50-CKB5-165 "ACCKee"</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1351,34 +1456,34 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>5205,00</t>
+          <t>8900,10</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>5205,00</t>
+          <t>8900,10</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB3-205</t>
+          <t>CKB6-TWN115150-75</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB3-205 sh00098</t>
+          <t>Расточная головка CKB6-TWN115150-75 "ACCKee"</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1393,34 +1498,34 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>19127,00</t>
+          <t>8529,30</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>19127,00</t>
+          <t>8529,30</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>BT50-45</t>
+          <t>BT50-CKB6-165</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>BESTE Штревель BT50-45 AC00601921</t>
+          <t>Оправка для расточных головок BT50-CKB6-165 "ACCKee"</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1430,39 +1535,39 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>931,00</t>
+          <t>8900,10</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2793,00</t>
+          <t>8900,10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>CKB4-TWN4154-50</t>
+          <t>BT50-CKB6-285</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB4-TWN4154-50 bh00015</t>
+          <t>Оправка для расточных головок BT50-CKB6-285 ACCKee</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1477,34 +1582,34 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>5682,00</t>
+          <t>13966,30</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>5682,00</t>
+          <t>13966,30</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>CKB5-TWN5372-60</t>
+          <t>CKB6-TWN89120-75</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB5-TWN5372-60 bh00001</t>
+          <t>Расточная головка CKB6-TWN89120-75 "ACCKee"</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1519,34 +1624,34 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>5883,00</t>
+          <t>5283,82</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>5883,00</t>
+          <t>5283,82</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-285</t>
+          <t>BT50-CKB6-205</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB6-285 db01991</t>
+          <t>Оправка для расточных головок BT50-CKB6-205 "ACCKee"</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1561,34 +1666,34 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>21498,00</t>
+          <t>10406,27</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>21498,00</t>
+          <t>10406,27</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB1-165</t>
+          <t>CKB6-TWN6890-75</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB1-165 sh00095</t>
+          <t>Расточная головка CKB6-TWN6890-75 "ACCKee"</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1603,34 +1708,34 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>16134,00</t>
+          <t>5032,21</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>16134,00</t>
+          <t>5032,21</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN115150-75</t>
+          <t>BT50-CKB6-125</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB6-TWN115150-75 bh00003</t>
+          <t>Оправка для расточных головок BT50-CKB6-125 "ACCKee"</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1645,34 +1750,34 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>17180,00</t>
+          <t>7667,77</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>17180,00</t>
+          <t>7667,77</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-165</t>
+          <t>BT50-CKB6-245</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка BT50-CKB6-165 sh00023</t>
+          <t>Оправка для расточных головок BT50-CKB6-245 "ACCKee"</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1687,34 +1792,34 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>17927,00</t>
+          <t>11090,89</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>17927,00</t>
+          <t>11090,89</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN89120-75</t>
+          <t>BT50-CKB4-245</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB6-TWN89120-75 bh00002</t>
+          <t>Оправка для расточных головок BT50-CKB4-245 "ACCKee"</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1729,12 +1834,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>10643,00</t>
+          <t>10406,27</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>10643,00</t>
+          <t>10406,27</t>
         </is>
       </c>
     </row>
@@ -2787,12 +2892,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>ООО «ВсеИнструменты.ру»</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -2829,17 +2934,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB3-TWN3242-43 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
+          <t>ACCKee Расточная головка CKB3-TWN3242-43 bh00018</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>5205,00</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>2720,11</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>5205,00</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2870,17 +2975,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB3-205 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB3-205 sh00098</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>19127,00</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>9995,48</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>19127,00</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2906,68 +3011,60 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CKB4-TWN4154-50</t>
+          <t>BT50-45</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB4-TWN4154-50 "ACCKee"</t>
+          <t>BESTE Штревель BT50-45 AC00601921</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2969,18</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>5682,00</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>4 430,00</t>
-        </is>
-      </c>
+          <t>931,00</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>2969.18</v>
+        <v>931</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>5682</v>
+        <v>931</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>2712.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CKB5-TWN5372-60</t>
+          <t>CKB4-TWN4154-50</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB5-TWN5372-60 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>3774,23</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>5883,00</t>
+          <t>ACCKee Расточная головка CKB4-TWN4154-50 bh00015</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>5682,00</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2969,18</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>4 730,00</t>
+          <t>4 430,00</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2976,150 +3073,154 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>3774.23</v>
+        <v>2969.18</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>5883</v>
+        <v>5682</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>2108.77</v>
+        <v>2712.82</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB5-245</t>
+          <t>CKB5-TWN5372-60</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB5-245 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>10406,27</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>ACCKee Расточная головка CKB5-TWN5372-60 bh00001</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>5883,00</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>3774,23</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>4 730,00</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>10406.27</v>
+        <v>3774.23</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>10406.27</v>
+        <v>5883</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0</v>
+        <v>2108.77</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB5-165</t>
+          <t>BT50-CKB6-285</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB5-165 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>8900,10</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>10 340,00</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB6-285 db01991</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>21498,00</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>13966,30</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>12 560,00</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО "ДОМИНИК"</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>8900.1</v>
+        <v>12560</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>10340</v>
+        <v>21498</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1439.9</v>
+        <v>8938</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN115150-75</t>
+          <t>BT50-CKB1-165</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN115150-75 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB1-165 sh00095</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>8529,30</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>17180,00</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>9 450,00</t>
-        </is>
-      </c>
+          <t>16134,00</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>8529.299999999999</v>
+        <v>16134</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>17180</v>
+        <v>16134</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>8650.700000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-165</t>
+          <t>CKB6-TWN115150-75</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-165 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>8900,10</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>17927,00</t>
+          <t>ACCKee Расточная головка CKB6-TWN115150-75 bh00003</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>17180,00</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>8529,30</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>10 340,00</t>
+          <t>9 450,00</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -3128,54 +3229,54 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>8900.1</v>
+        <v>8529.299999999999</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>17927</v>
+        <v>17180</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>9026.9</v>
+        <v>8650.700000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-285</t>
+          <t>BT50-CKB6-165</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-285 ACCKee</t>
+          <t>ACCKee Оправка BT50-CKB6-165 sh00023</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>13966,30</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>21498,00</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>12 560,00</t>
+          <t>17927,00</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>8900,10</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>10 340,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ООО "ДОМИНИК"</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>12560</v>
+        <v>8900.1</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>21498</v>
+        <v>17927</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>8938</v>
+        <v>9026.9</v>
       </c>
     </row>
     <row r="11">
@@ -3186,17 +3287,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN89120-75 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+          <t>ACCKee Расточная головка CKB6-TWN89120-75 bh00002</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>10643,00</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>5283,82</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>10643,00</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -3222,60 +3323,56 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-205</t>
+          <t>BT50-CKB5-245</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-205 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
+          <t>Оправка для расточных головок BT50-CKB5-245 "ACCKee"</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>10406,27</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>9 380,00</t>
-        </is>
-      </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>ООО "ДОМИНИК"</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>9380</v>
+        <v>10406.27</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>10406.27</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1026.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN6890-75</t>
+          <t>BT50-CKB5-165</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN6890-75 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>5032,21</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
+          <t>Оправка для расточных головок BT50-CKB5-165 "ACCKee"</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>8900,10</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>6 300,00</t>
+          <t>10 340,00</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3284,35 +3381,35 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>5032.21</v>
+        <v>8900.1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>6300</v>
+        <v>10340</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>1267.79</v>
+        <v>1439.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-125</t>
+          <t>BT50-CKB6-205</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-125 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>7667,77</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>Оправка для расточных головок BT50-CKB6-205 "ACCKee"</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>10406,27</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>6 890,00</t>
+          <t>9 380,00</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3321,153 +3418,161 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>6890</v>
+        <v>9380</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>7667.77</v>
+        <v>10406.27</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>777.7700000000004</v>
+        <v>1026.27</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-245</t>
+          <t>CKB6-TWN6890-75</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-245 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>11090,89</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>9 990,00</t>
+          <t>Расточная головка CKB6-TWN6890-75 "ACCKee"</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>5032,21</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>6 300,00</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>ООО "ДОМИНИК"</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>9990</v>
+        <v>5032.21</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>11090.89</v>
+        <v>6300</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1100.889999999999</v>
+        <v>1267.79</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB4-245</t>
+          <t>BT50-CKB6-125</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB4-245 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>10406,27</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>16 912,00</t>
+          <t>Оправка для расточных головок BT50-CKB6-125 "ACCKee"</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>7667,77</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>6 890,00</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО "ДОМИНИК"</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>10406.27</v>
+        <v>6890</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>16912</v>
+        <v>7667.77</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>6505.73</v>
+        <v>777.7700000000004</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BT50-45</t>
+          <t>BT50-CKB6-245</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>BESTE Штревель BT50-45 AC00601921</t>
+          <t>Оправка для расточных головок BT50-CKB6-245 "ACCKee"</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>931,00</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>11090,89</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>9 990,00</t>
+        </is>
+      </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>ООО "ДОМИНИК"</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>931</v>
+        <v>9990</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>931</v>
+        <v>11090.89</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0</v>
+        <v>1100.889999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB1-165</t>
+          <t>BT50-CKB4-245</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB1-165 sh00095</t>
+          <t>Оправка для расточных головок BT50-CKB4-245 "ACCKee"</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>16134,00</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
+          <t>10406,27</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>16 912,00</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>16134</v>
+        <v>10406.27</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>16134</v>
+        <v>16912</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>6505.73</v>
       </c>
     </row>
     <row r="19">
@@ -3652,42 +3757,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ООО «ВсеИнструменты.ру»</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>17065</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Лидер по количеству минимальных цен</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B3" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C3" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D3" s="3" t="n">
         <v>66921.59</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Лидер по количеству минимальных цен</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>17065</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Лидер по количеству минимальных цен</t>
         </is>
@@ -3784,7 +3889,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>61546.60999999999</v>
+        <v>61546.61</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Add OCR support for scanned PDFs
</commit_message>
<xml_diff>
--- a/Сравнение_КП_959777517.xlsx
+++ b/Сравнение_КП_959777517.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сравнение КП'!$A$1:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Позиции КП'!$A$1:$H$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Конкурентная карта'!$A$1:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Конкурентная карта'!$A$1:$I$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Итоги поставщиков'!$A$1:$E$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Заключение'!$A$1:$B$8</definedName>
   </definedNames>
@@ -552,12 +552,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>122 072,00 ₽</t>
+          <t>120 048,30</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -567,17 +567,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>самовывоз</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>от 5 до 7 раб.дн.</t>
+          <t>срок резервирования товара 3 рабочих дня</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>полная оплата счета, акцепт в течение 3 рабочих дней</t>
+          <t>товар отпускается по факту прихода денег на р/с Поставщика</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -587,12 +587,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>3 рабочих дня с даты выставления счета (26 марта 2026 года)</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>ACCKee, BESTE</t>
+          <t>ACCKee</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Доставка - самовывоз из г. Челябинск, ул. Комарова, д. 110. Гарантия не указана. Срок поставки от 5 до 7 рабочих дней. Оплата полная, акцепт оферты в течение 3 рабочих дней.</t>
+          <t>Оплата означает согласие с условиями поставки. Уведомление об оплате обязательно, иначе наличие товара не гарантируется.</t>
         </is>
       </c>
     </row>
@@ -612,12 +612,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>120 048,30</t>
+          <t>122 072,00 ₽</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -627,42 +627,42 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>самовывоз</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>от 5 до 7 раб.дн.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>полная оплата счета, акцепт в течение 3 рабочих дней</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>срок резервирования товара 3 рабочих дня</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>товар отпускается по факту прихода денег на р/с Поставщика</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>3 рабочих дня с даты выставления счета (26 марта 2026 года)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>ACCKee, BESTE</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>ACCKee</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Оплата означает согласие с условиями поставки. Уведомление об оплате обязательно. Гарантия и срок действия КП не указаны. Доставка не указана.</t>
+          <t>Доставка - самовывоз из г. Челябинск, ул. Комарова, д. 110. Гарантия не указана. Срок поставки от 5 до 7 рабочих дней. Оплата полная, акцепт оферты в течение 3 рабочих дней.</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Доставка не указана, гарантия не указана, производитель и страна не указаны.</t>
+          <t>Доставка не указана. Гарантия не указана. Производитель и страна происхождения не указаны.</t>
         </is>
       </c>
     </row>
@@ -796,12 +796,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB3-TWN3242-43 bh00018</t>
+          <t>Расточная головка CKB3-TWN3242-43</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -821,29 +821,29 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>5205,00</t>
+          <t>2720,11</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>5205,00</t>
+          <t>2720,11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB3-205 sh00098</t>
+          <t>Оправка для расточных головок BT50-CKB3-205</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -863,39 +863,39 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>19127,00</t>
+          <t>9995,48</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>19127,00</t>
+          <t>9995,48</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>BT50-45</t>
+          <t>CKB4-TWN4154-50</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BESTE Штревель BT50-45 AC00601921</t>
+          <t>Расточная головка CKB4-TWN4154-50</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -905,39 +905,39 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>931,00</t>
+          <t>2969,18</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2793,00</t>
+          <t>2969,18</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>CKB4-TWN4154-50</t>
+          <t>CKB5-TWN5372-60</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB4-TWN4154-50 bh00015</t>
+          <t>Расточная головка CKB5-TWN5372-60</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -947,39 +947,39 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>5682,00</t>
+          <t>3774,23</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>5682,00</t>
+          <t>не указано</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>CKB5-TWN5372-60</t>
+          <t>BT50-CKB5-245</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB5-TWN5372-60 bh00001</t>
+          <t>Оправка для расточных головок BT50-CKB5-245</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -989,39 +989,39 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>5883,00</t>
+          <t>406,27</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>5883,00</t>
+          <t>4062,7</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-285</t>
+          <t>СКВ5-165</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB6-285 db01991</t>
+          <t>Оправка для расточных головок ВТ50-СКВ5-165</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1031,39 +1031,39 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>21498,00</t>
+          <t>900,10</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>21498,00</t>
+          <t>7200,8</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB1-165</t>
+          <t>CKB6-TWN115150-75</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB1-165 sh00095</t>
+          <t>Расточная головка CKB6-TWN115150-75</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1073,39 +1073,39 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>16134,00</t>
+          <t>8529,30</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>16134,00</t>
+          <t>не указано</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN115150-75</t>
+          <t>BT50-CKB6-165</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB6-TWN115150-75 bh00003</t>
+          <t>Оправка для расточных головок BT50-CKB6-165</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1115,39 +1115,39 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>17180,00</t>
+          <t>900,10</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>17180,00</t>
+          <t>не указано</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-165</t>
+          <t>BT50-CKB6-285</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка BT50-CKB6-165 sh00023</t>
+          <t>Оправка для расточных головок BT50-CKB6-285</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1157,29 +1157,29 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>17927,00</t>
+          <t>13966,30</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>17927,00</t>
+          <t>13966,30</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB6-TWN89120-75 bh00002</t>
+          <t>Расточная головка CKB6-TWN89120-75</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1199,24 +1199,24 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>10643,00</t>
+          <t>5283,82</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>10643,00</t>
+          <t>5283,82</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1226,12 +1226,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>CKB3-TWN3242-43</t>
+          <t>BT50-CKB6-205</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB3-TWN3242-43 "ACCKee"</t>
+          <t>Оправка для расточных головок BT50-CKB6-205</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1241,24 +1241,24 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2720,11</t>
+          <t>406,27</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2720,11</t>
+          <t>4062,7</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1268,12 +1268,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB3-205</t>
+          <t>CKB6-TWN6890-75</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB3-205 "ACCKee"</t>
+          <t>Расточная головка CKB6-TWN6890-75</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1283,24 +1283,24 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>9995,48</t>
+          <t>5032,21</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>9995,48</t>
+          <t>5032,21</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>CKB4-TWN4154-50</t>
+          <t>BT50-CKB6-125</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB4-TWN4154-50 "ACCKee"</t>
+          <t>Оправка для расточных головок BT50-CKB6-125</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1325,24 +1325,24 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2969,18</t>
+          <t>7667,77</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2969,18</t>
+          <t>7667,77</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>CKB5-TWN5372-60</t>
+          <t>BT50-CKB6-245</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB5-TWN5372-60 "ACCKee"</t>
+          <t>Оправка для расточных головок BT50-CKB6-245</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1367,24 +1367,24 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>3774,23</t>
+          <t>11090,89</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>3774,23</t>
+          <t>11090,89</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>doc01972620260520192040.pdf</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1394,12 +1394,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB5-245</t>
+          <t>BT50-CKB4-245</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB5-245 "ACCKee"</t>
+          <t>Оправка для расточных головок BT50-CKB4-245</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>не указано</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1426,22 +1426,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB5-165</t>
+          <t>CKB3-TWN3242-43</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB5-165 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB3-TWN3242-43 bh00018</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1456,34 +1456,34 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>8900,10</t>
+          <t>5205,00</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>8900,10</t>
+          <t>5205,00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN115150-75</t>
+          <t>BT50-CKB3-205</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN115150-75 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB3-205 sh00098</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1498,34 +1498,34 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>8529,30</t>
+          <t>19127,00</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>8529,30</t>
+          <t>19127,00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-165</t>
+          <t>BT50-45</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-165 "ACCKee"</t>
+          <t>BESTE Штревель BT50-45 AC00601921</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1535,39 +1535,39 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>8900,10</t>
+          <t>931,00</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>8900,10</t>
+          <t>2793,00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-285</t>
+          <t>CKB4-TWN4154-50</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-285 ACCKee</t>
+          <t>ACCKee Расточная головка CKB4-TWN4154-50 bh00015</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1582,34 +1582,34 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>13966,30</t>
+          <t>5682,00</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>13966,30</t>
+          <t>5682,00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN89120-75</t>
+          <t>CKB5-TWN5372-60</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN89120-75 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB5-TWN5372-60 bh00001</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1624,34 +1624,34 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>5283,82</t>
+          <t>5883,00</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>5283,82</t>
+          <t>5883,00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-205</t>
+          <t>BT50-CKB6-285</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-205 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB6-285 db01991</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1666,34 +1666,34 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>10406,27</t>
+          <t>21498,00</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>10406,27</t>
+          <t>21498,00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN6890-75</t>
+          <t>BT50-CKB1-165</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN6890-75 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB1-165 sh00095</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1708,34 +1708,34 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>5032,21</t>
+          <t>16134,00</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>5032,21</t>
+          <t>16134,00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-125</t>
+          <t>CKB6-TWN115150-75</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-125 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB6-TWN115150-75 bh00003</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1750,34 +1750,34 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>7667,77</t>
+          <t>17180,00</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>7667,77</t>
+          <t>17180,00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-245</t>
+          <t>BT50-CKB6-165</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-245 "ACCKee"</t>
+          <t>ACCKee Оправка BT50-CKB6-165 sh00023</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1792,34 +1792,34 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>11090,89</t>
+          <t>17927,00</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>11090,89</t>
+          <t>17927,00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>КП_Вольфстар_ООО_Счет_на_оплату_№_856_от_26_марта_2026_г_1.pdf</t>
+          <t>КП_Все_инструменты_ООО_Счет_на_оплату_№2603_453438_40628.pdf</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB4-245</t>
+          <t>CKB6-TWN89120-75</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB4-245 "ACCKee"</t>
+          <t>ACCKee Расточная головка CKB6-TWN89120-75 bh00002</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1834,12 +1834,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>10406,27</t>
+          <t>10643,00</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>10406,27</t>
+          <t>10643,00</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2892,12 +2892,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>ООО «ВсеИнструменты.ру»</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -2934,17 +2934,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB3-TWN3242-43 bh00018</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+          <t>Расточная головка CKB3-TWN3242-43</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2720,11</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>5205,00</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>2720,11</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2975,17 +2975,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB3-205 sh00098</t>
+          <t>Оправка для расточных головок BT50-CKB3-205</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>9995,48</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>19127,00</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>9995,48</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -3011,60 +3011,68 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BT50-45</t>
+          <t>CKB4-TWN4154-50</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>BESTE Штревель BT50-45 AC00601921</t>
+          <t>Расточная головка CKB4-TWN4154-50</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>931,00</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>2969,18</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>5682,00</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>4 430,00</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>931</v>
+        <v>2969.18</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>931</v>
+        <v>5682</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0</v>
+        <v>2712.82</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CKB4-TWN4154-50</t>
+          <t>CKB5-TWN5372-60</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB4-TWN4154-50 bh00015</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>5682,00</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>2969,18</t>
+          <t>Расточная головка CKB5-TWN5372-60</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>3774,23</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>5883,00</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>4 430,00</t>
+          <t>4 730,00</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -3073,154 +3081,146 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>2969.18</v>
+        <v>3774.23</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>5682</v>
+        <v>5883</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>2712.82</v>
+        <v>2108.77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>CKB5-TWN5372-60</t>
+          <t>BT50-CKB5-245</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB5-TWN5372-60 bh00001</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>5883,00</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>3774,23</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>4 730,00</t>
-        </is>
-      </c>
+          <t>Оправка для расточных головок BT50-CKB5-245</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>406,27</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>3774.23</v>
+        <v>406.27</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>5883</v>
+        <v>406.27</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>2108.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-285</t>
+          <t>СКВ5-165</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB6-285 db01991</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>21498,00</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>13966,30</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>12 560,00</t>
-        </is>
-      </c>
+          <t>Оправка для расточных головок ВТ50-СКВ5-165</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>900,10</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>ООО "ДОМИНИК"</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>12560</v>
+        <v>900.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>21498</v>
+        <v>900.1</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>8938</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB1-165</t>
+          <t>CKB6-TWN115150-75</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка для расточных головок BT50-CKB1-165 sh00095</t>
+          <t>Расточная головка CKB6-TWN115150-75</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>16134,00</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>8529,30</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>17180,00</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>9 450,00</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>ООО «ВсеИнструменты.ру»</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>16134</v>
+        <v>8529.299999999999</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>16134</v>
+        <v>17180</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0</v>
+        <v>8650.700000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN115150-75</t>
+          <t>BT50-CKB6-165</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB6-TWN115150-75 bh00003</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>17180,00</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>8529,30</t>
+          <t>Оправка для расточных головок BT50-CKB6-165</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>900,10</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>17927,00</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>9 450,00</t>
+          <t>10 340,00</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -3229,54 +3229,54 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>8529.299999999999</v>
+        <v>900.1</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>17180</v>
+        <v>17927</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>8650.700000000001</v>
+        <v>17026.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-165</t>
+          <t>BT50-CKB6-285</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Оправка BT50-CKB6-165 sh00023</t>
+          <t>Оправка для расточных головок BT50-CKB6-285</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>17927,00</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>8900,10</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>10 340,00</t>
+          <t>13966,30</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>21498,00</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>12 560,00</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО "ДОМИНИК"</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>8900.1</v>
+        <v>12560</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>17927</v>
+        <v>21498</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>9026.9</v>
+        <v>8938</v>
       </c>
     </row>
     <row r="11">
@@ -3287,17 +3287,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ACCKee Расточная головка CKB6-TWN89120-75 bh00002</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
+          <t>Расточная головка CKB6-TWN89120-75</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>5283,82</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>10643,00</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>5283,82</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -3323,56 +3323,60 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB5-245</t>
+          <t>BT50-CKB6-205</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB5-245 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>10406,27</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+          <t>Оправка для расточных головок BT50-CKB6-205</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>406,27</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>9 380,00</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>10406.27</v>
+        <v>406.27</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>10406.27</v>
+        <v>9380</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0</v>
+        <v>8973.73</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB5-165</t>
+          <t>CKB6-TWN6890-75</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB5-165 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>8900,10</t>
-        </is>
-      </c>
+          <t>Расточная головка CKB6-TWN6890-75</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>5032,21</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>10 340,00</t>
+          <t>6 300,00</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3381,35 +3385,35 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>8900.1</v>
+        <v>5032.21</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>10340</v>
+        <v>6300</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>1439.9</v>
+        <v>1267.79</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-205</t>
+          <t>BT50-CKB6-125</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-205 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>10406,27</t>
-        </is>
-      </c>
+          <t>Оправка для расточных головок BT50-CKB6-125</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>7667,77</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>9 380,00</t>
+          <t>6 890,00</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3418,161 +3422,153 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>9380</v>
+        <v>6890</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>10406.27</v>
+        <v>7667.77</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>1026.27</v>
+        <v>777.7700000000004</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CKB6-TWN6890-75</t>
+          <t>BT50-CKB6-245</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Расточная головка CKB6-TWN6890-75 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>5032,21</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>6 300,00</t>
+          <t>Оправка для расточных головок BT50-CKB6-245</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>11090,89</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>9 990,00</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО "ДОМИНИК"</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>5032.21</v>
+        <v>9990</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>6300</v>
+        <v>11090.89</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1267.79</v>
+        <v>1100.889999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-125</t>
+          <t>BT50-CKB4-245</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-125 "ACCKee"</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>7667,77</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>6 890,00</t>
+          <t>Оправка для расточных головок BT50-CKB4-245</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>10406,27</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>16 912,00</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>ООО "ДОМИНИК"</t>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>6890</v>
+        <v>10406.27</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>7667.77</v>
+        <v>16912</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>777.7700000000004</v>
+        <v>6505.73</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB6-245</t>
+          <t>BT50-45</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB6-245 "ACCKee"</t>
+          <t>BESTE Штревель BT50-45 AC00601921</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>11090,89</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>9 990,00</t>
-        </is>
-      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>931,00</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>ООО "ДОМИНИК"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>9990</v>
+        <v>931</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>11090.89</v>
+        <v>931</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>1100.889999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BT50-CKB4-245</t>
+          <t>BT50-CKB1-165</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Оправка для расточных головок BT50-CKB4-245 "ACCKee"</t>
+          <t>ACCKee Оправка для расточных головок BT50-CKB1-165 sh00095</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>10406,27</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>16 912,00</t>
-        </is>
-      </c>
+          <t>16134,00</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+          <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>10406.27</v>
+        <v>16134</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>16912</v>
+        <v>16134</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>6505.73</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -3644,19 +3640,19 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>RDH-D151-211-80L</t>
+          <t>BT50-CKB5-165</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>RDH-D151-211-80L черновая расточная головка</t>
+          <t>BT50-CKB5-165 оправка для расточных систем</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>14 250,00</t>
+          <t>10 340,00</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -3665,10 +3661,10 @@
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>14250</v>
+        <v>10340</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>14250</v>
+        <v>10340</v>
       </c>
       <c r="I21" s="2" t="n">
         <v>0</v>
@@ -3677,19 +3673,19 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BT50-DM32-300</t>
+          <t>RDH-D151-211-80L</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>BT50-DM32-300 оправка для расточных систем</t>
+          <t>RDH-D151-211-80L черновая расточная головка</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>20 482,00</t>
+          <t>14 250,00</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -3698,17 +3694,50 @@
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>20482</v>
+        <v>14250</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>20482</v>
+        <v>14250</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>BT50-DM32-300</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>BT50-DM32-300 оправка для расточных систем</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>20 482,00</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ДОМИНИК"</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>20482</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>20482</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:I23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3757,42 +3786,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>41327.86</v>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Лидер по количеству минимальных цен</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ООО «ВсеИнструменты.ру»</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B3" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D3" s="2" t="n">
         <v>17065</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Лидер по количеству минимальных цен</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Общество с ограниченной ответственностью "ВОЛЬФСТАР"</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>66921.59</v>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Лидер по количеству минимальных цен</t>
         </is>
@@ -3811,7 +3840,7 @@
         <v>9</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>93832</v>
+        <v>94792</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -3867,7 +3896,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -3889,7 +3918,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>61546.61</v>
+        <v>76054.17</v>
       </c>
     </row>
     <row r="6">

</xml_diff>